<commit_message>
This Swag Labs file
</commit_message>
<xml_diff>
--- a/testdata/SwagLabsData.xlsx
+++ b/testdata/SwagLabsData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bba62b6a9631ba18/MyLearn/Python/PythonEcomm/testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{CFB4E50B-4E1A-455D-9E0F-E1E7818B4443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05DA313C-2F92-4E8B-A89A-E31DFA0ACE68}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{CFB4E50B-4E1A-455D-9E0F-E1E7818B4443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4C9E484-59DA-4D54-A3F2-4EB08D5AC6F8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7EE64AE-36E7-43D4-89CD-0EF19ADB0C9E}"/>
   </bookViews>
@@ -82,7 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,6 +96,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -118,11 +123,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C860AB60-B720-45B1-B2A0-775540D5671A}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -505,6 +511,22 @@
         <v>11</v>
       </c>
     </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>